<commit_message>
Fill Social Listening survey results into 15/10 report and tracking workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0113oF5reXaFkT1cmVdQS56Z
</commit_message>
<xml_diff>
--- a/reports/Social_Listening_COKI_Theo_doi.xlsx
+++ b/reports/Social_Listening_COKI_Theo_doi.xlsx
@@ -550,272 +550,944 @@
         <f>IF(E2="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
+      <c r="B2" s="3" t="n">
+        <v>46310</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Fanpage</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Comment dưới bài QC đa tròng (đăng 30/9): hỏi có kính lão 1,2 độ không</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>https://business.facebook.com/latest/inbox/facebook?asset_id=190065937527579&amp;thread_type=FB_PAGE_POST&amp;selected_item_id=1346020201932141</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Trung tính</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Mẫu mã</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>1 cảm xúc</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Ngày ≈ ("8 giờ"). Trang trả lời câu mẫu "đã inbox"</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2">
         <f>IF(E3="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
+      <c r="B3" s="3" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Fanpage</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Bài "Deal xinh rộn ràng" (3/10): khách hỏi ưu đãi giảm 200K cho khách mới; kể hôm qua đến cửa hàng nhân viên nói đã hết chương trình</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>https://business.facebook.com/latest/inbox/facebook?asset_id=190065937527579&amp;thread_type=FB_PAGE_POST&amp;selected_item_id=1357437214123773</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Tiêu cực</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Khuyến mãi</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Chưa</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>1 cảm xúc</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Ngày ≈. Trang chỉ trả lời câu mẫu, chưa nhắc đến phàn nàn</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2">
         <f>IF(E4="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
+      <c r="B4" s="3" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Fanpage</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Bài "Con tăng độ cận" (29/9): hỏi giá</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>https://business.facebook.com/latest/inbox/facebook?asset_id=190065937527579&amp;thread_type=FB_PAGE_POST&amp;selected_item_id=1358110050723156</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Trung tính</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Giá</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Ngày ≈ ("23 giờ"). Câu mẫu "đã inbox"</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2">
         <f>IF(E5="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="n"/>
-      <c r="K5" s="2" t="n"/>
-      <c r="L5" s="2" t="n"/>
+      <c r="B5" s="3" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Fanpage</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Bài "Con mới 3 tuổi…" (22/8): muốn được tư vấn</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>https://business.facebook.com/latest/inbox/facebook?asset_id=190065937527579&amp;thread_type=FB_PAGE_POST&amp;selected_item_id=1316935531507275</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Trung tính</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Dịch vụ</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Ngày ≈. Câu mẫu "đã inbox"</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2">
         <f>IF(E6="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
+      <c r="B6" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Fanpage</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Bài QC tròng lọc ánh sáng xanh (29/8): xin giá</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>https://business.facebook.com/latest/inbox/facebook?asset_id=190065937527579&amp;thread_type=FB_PAGE_POST&amp;selected_item_id=1314258838441611</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Trung tính</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Giá</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Chưa</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Ngày ≈ ("6 ngày"). Chưa thấy trang trả lời trực tiếp</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2">
         <f>IF(E7="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
+      <c r="B7" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Fanpage</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Bài "Ra đường phải nheo mắt" (30/9): xin giá</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>https://business.facebook.com/latest/inbox/facebook?asset_id=190065937527579&amp;thread_type=FB_PAGE_POST&amp;selected_item_id=1343448765522618</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Trung tính</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Giá</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Ngày ≈. Câu mẫu "đã inbox"</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2">
         <f>IF(E8="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
+      <c r="B8" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Fanpage</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Ảnh trong bài 6/10: xin giá mẫu gọng</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>https://business.facebook.com/latest/inbox/facebook?asset_id=190065937527579&amp;thread_type=FB_PAGE_POST&amp;selected_item_id=1349680864899408</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Trung tính</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Giá</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Ngày ≈. Đã báo giá 350K</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2">
         <f>IF(E9="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="n"/>
-      <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="n"/>
+      <c r="B9" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Fanpage</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Bài tròng lọc ánh sáng xanh: xin giá</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>https://business.facebook.com/latest/inbox/facebook?asset_id=190065937527579&amp;thread_type=FB_PAGE_POST&amp;selected_item_id=1314258838441611</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Trung tính</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Giá</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Ngày ≈ 02–08/10 ("1 tuần"), có thể ngoài kỳ. Câu mẫu "đã inbox"</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2">
         <f>IF(E10="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="n"/>
+      <c r="B10" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Fanpage</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Bài tròng lọc ánh sáng xanh: hỏi giá</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>https://business.facebook.com/latest/inbox/facebook?asset_id=190065937527579&amp;thread_type=FB_PAGE_POST&amp;selected_item_id=1314258838441611</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Trung tính</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Giá</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Ngày ≈ 02–08/10, có thể ngoài kỳ. Có 1 phản hồi</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2">
         <f>IF(E11="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="n"/>
-      <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="n"/>
+      <c r="B11" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Fanpage</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Bài tròng lọc ánh sáng xanh: xin giá</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>https://business.facebook.com/latest/inbox/facebook?asset_id=190065937527579&amp;thread_type=FB_PAGE_POST&amp;selected_item_id=1314258838441611</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Trung tính</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Giá</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Ngày ≈ 02–08/10, có thể ngoài kỳ. Có 1 phản hồi</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2">
         <f>IF(E12="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="n"/>
-      <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="n"/>
+      <c r="B12" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Fanpage</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Bài "Ra đường phải nheo mắt": hỏi kính chống lóa đi đêm</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>https://business.facebook.com/latest/inbox/facebook?asset_id=190065937527579&amp;thread_type=FB_PAGE_POST&amp;selected_item_id=1343448765522618</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Trung tính</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Mẫu mã</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Ngày ≈ 02–08/10, có thể ngoài kỳ. Có 1 phản hồi</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2">
         <f>IF(E13="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
-      <c r="J13" s="2" t="n"/>
-      <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="n"/>
+      <c r="B13" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Fanpage</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Bài "Cận 4–5 độ" (30/9): xin giá tròng đổi màu</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>https://business.facebook.com/latest/inbox/facebook?asset_id=190065937527579&amp;thread_type=FB_PAGE_POST&amp;selected_item_id=1347270231807138</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Trung tính</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Giá</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Ngày ≈ 08/10 ("1 tuần"). Câu mẫu "đã inbox"</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2">
         <f>IF(E14="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="n"/>
-      <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="n"/>
+      <c r="B14" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Kính mắt COKI</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>COKI Thủy Nguyên – 1 sao: đo mắt 2 lần, cả 2 lần đến cắt kính đều báo hết tròng; rất thất vọng, có thể không quay lại</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps – bài mới nhất (cửa hàng Thủy Nguyên)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Tiêu cực</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Dịch vụ</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Chưa</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Ngày không chính xác ("một tuần trước"), có thể ngoài kỳ. Cửa hàng chưa trả lời</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2">
         <f>IF(E15="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
-      <c r="J15" s="2" t="n"/>
-      <c r="K15" s="2" t="n"/>
-      <c r="L15" s="2" t="n"/>
+      <c r="B15" s="3" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Kính mắt COKI / kính COKI</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Video giới thiệu tròng Essilor Eyezen (@kinhmatcoki)</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Xem trong báo cáo khảo sát</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Trung tính</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Mẫu mã</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>303 xem, 2 tim, 0 bình luận</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Lượt chia sẻ không lấy được</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2">
         <f>IF(E16="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="n"/>
-      <c r="K16" s="2" t="n"/>
-      <c r="L16" s="2" t="n"/>
+      <c r="B16" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Kính mắt COKI</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Bài ảnh: gọng mới về (@kinhmatcoki)</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Xem trong báo cáo khảo sát</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Trung tính</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Mẫu mã</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>363 xem, 1 tim, 0 bình luận</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Lượt chia sẻ không lấy được</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2">
         <f>IF(E17="","",ROW()-1)</f>
         <v/>
       </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
-      <c r="J17" s="2" t="n"/>
-      <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="n"/>
+      <c r="B17" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Kính mắt COKI</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Bài ảnh: deal Tháng của nàng (@kinhmatcoki)</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Xem trong báo cáo khảo sát</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Trung tính</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Khuyến mãi</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>365 xem, 0 tim, 0 bình luận</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Lượt chia sẻ không lấy được</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2">
@@ -9076,7 +9748,9 @@
           <t>Từ ngày</t>
         </is>
       </c>
-      <c r="B2" s="5" t="n"/>
+      <c r="B2" s="5" t="n">
+        <v>46300</v>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>← nhập ngày đầu kỳ</t>
@@ -9089,7 +9763,9 @@
           <t>Đến ngày</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n"/>
+      <c r="B3" s="5" t="n">
+        <v>46310</v>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>← nhập ngày cuối kỳ</t>
@@ -9207,7 +9883,6 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
@@ -9293,8 +9968,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
@@ -9380,7 +10053,6 @@
         <v/>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>

</xml_diff>